<commit_message>
update mobidam schema and export for initial filling
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_mobidam.xlsx
+++ b/ckanext/lhm/schemas/template_mobidam.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckan-helm\lhmchart\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F161BC8A-2A62-4834-972A-2BE9F8D16D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7159ED12-CB8C-476C-B6FF-3AB637AF6648}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="21792" windowHeight="11772" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
+    <workbookView xWindow="1248" yWindow="1536" windowWidth="21792" windowHeight="10440" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadaten" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="235">
   <si>
     <t>nein</t>
   </si>
@@ -764,7 +764,10 @@
     <t>Bedeutung</t>
   </si>
   <si>
-    <t>1.2.5.</t>
+    <t>1.2.5-demo-2</t>
+  </si>
+  <si>
+    <t>k.A.</t>
   </si>
 </sst>
 </file>
@@ -2378,20 +2381,38 @@
       <c r="E5" s="2" t="s">
         <v>147</v>
       </c>
+      <c r="F5" s="4" t="s">
+        <v>234</v>
+      </c>
       <c r="G5" s="3" t="s">
         <v>117</v>
       </c>
+      <c r="H5" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="I5" s="3" t="s">
         <v>178</v>
       </c>
+      <c r="J5" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="K5" s="3" t="s">
         <v>173</v>
       </c>
+      <c r="L5" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="N5" s="3" t="s">
         <v>165</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>92</v>
+      </c>
+      <c r="Q5" s="2" t="s">
+        <v>234</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>98</v>
@@ -2512,9 +2533,17 @@
       <c r="C9" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E9" s="1"/>
+      <c r="D9" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>234</v>
+      </c>
       <c r="G9" s="3" t="s">
         <v>121</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>234</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>86</v>
@@ -2578,6 +2607,9 @@
         <v>135</v>
       </c>
       <c r="E12" s="1"/>
+      <c r="G12" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="K12" s="15"/>
       <c r="U12" s="2" t="s">
         <v>199</v>
@@ -2792,7 +2824,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="7WMZ1mDUyvhL4UpKWt0nfcgkaCP0BpTdJaHaP4ZqioaIBj5Otagyz61Gxt0x4SOLv8AaGVTwJsZOUhjfi81XSw==" saltValue="yvb7SbXdXcRytveSJfy99Q==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="tHqX5IzvbVLg/sih/nBV5JSwd94s+M1ONwVfux2ZHcdTBVghR6J7oMB8B1Yk4AmxuhkvPBQYZbiiYSYwTUZ4dg==" saltValue="MPlADdkP375xV3lHONZ/Xg==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update excel mobidem template version number
</commit_message>
<xml_diff>
--- a/ckanext/lhm/schemas/template_mobidam.xlsx
+++ b/ckanext/lhm/schemas/template_mobidam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\home\mb\p2\ckanext-lhm\ckanext\lhm\schemas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C34CCE-D4CC-40C7-8908-AAB439508000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE23BF3E-CD69-4CBD-9F1F-881EA0E08A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="871" xr2:uid="{EFAD0BDA-2C19-4F99-80E8-84599936D919}"/>
   </bookViews>
@@ -767,7 +767,7 @@
     <t>k.A.</t>
   </si>
   <si>
-    <t>1.3.1.</t>
+    <t>1.3.1-demo</t>
   </si>
 </sst>
 </file>

</xml_diff>